<commit_message>
Lead table: green/red/blue row colors for Квал/Не квал/Недозвон
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018zXrhLFn975wKHPSJbBzzV
</commit_message>
<xml_diff>
--- a/leads-sheet/MEDELA-лиды.xlsx
+++ b/leads-sheet/MEDELA-лиды.xlsx
@@ -89,17 +89,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8E6C9"/>
+        <fgColor rgb="00B6D7A8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7DA"/>
+        <fgColor rgb="00EA9999"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFE8B3"/>
+        <fgColor rgb="00A4C2F4"/>
       </patternFill>
     </fill>
   </fills>
@@ -162,21 +162,21 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00C8E6C9"/>
+          <fgColor rgb="00B6D7A8"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00F8D7DA"/>
+          <fgColor rgb="00EA9999"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00FFE8B3"/>
+          <fgColor rgb="00A4C2F4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -650,7 +650,7 @@
         <v/>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46314</v>
+        <v>46317</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -16292,7 +16292,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>4. Строка окрасится по статусу: зелёный — квал, красный — не квал, жёлтый — недозвон.</t>
+          <t>4. Строка окрасится по статусу: зелёный — квал, красный — не квал, синий — недозвон.</t>
         </is>
       </c>
     </row>

</xml_diff>